<commit_message>
feat: ActionData 재정의, UserData 주입
</commit_message>
<xml_diff>
--- a/BADesign/Excel/Player.xlsx
+++ b/BADesign/Excel/Player.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>Client</t>
   </si>
@@ -56,32 +56,44 @@
     <t>Name</t>
   </si>
   <si>
-    <t>ActionType</t>
-  </si>
-  <si>
-    <t>CoolTime</t>
-  </si>
-  <si>
-    <t>ConsumeStamina</t>
-  </si>
-  <si>
-    <t>기본공격 1타</t>
-  </si>
-  <si>
-    <t>가드</t>
-  </si>
-  <si>
-    <t>전력질주</t>
-  </si>
-  <si>
-    <t>구르기</t>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>StaminaCost</t>
+  </si>
+  <si>
+    <t>MinRequiredStamina</t>
+  </si>
+  <si>
+    <t>LightAttack</t>
+  </si>
+  <si>
+    <t>Attack</t>
+  </si>
+  <si>
+    <t>HeavyAttack</t>
+  </si>
+  <si>
+    <t>Guard</t>
+  </si>
+  <si>
+    <t>Defence</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Movement</t>
+  </si>
+  <si>
+    <t>DodgeRoll</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -99,12 +111,21 @@
       <name val="&quot;맑은 고딕&quot;"/>
     </font>
     <font>
-      <color theme="1"/>
+      <sz val="9.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="&quot;\0022맑은 고딕\0022&quot;"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;\0022맑은 고딕\0022&quot;"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -115,12 +136,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF595959"/>
         <bgColor rgb="FF595959"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBFBFBF"/>
-        <bgColor rgb="FFBFBFBF"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -157,11 +172,17 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,116 +528,139 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="5" max="5" width="25.5"/>
+    <col customWidth="1" min="6" max="6" width="27.0"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C1" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="D1" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="E1" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="F1" s="1">
+      <c r="B1" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C1" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="D1" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E1" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="F1" s="4">
         <v>1.0</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="2">
+      <c r="A3" s="6"/>
+      <c r="B3" s="5">
         <v>10001.0</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>5.0</v>
+      <c r="D3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="5">
+        <v>15.0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3"/>
-      <c r="B4" s="2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5">
+        <v>10002.0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="5">
+        <v>30.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6"/>
+      <c r="B5" s="5">
         <v>10011.0</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="5">
+      <c r="C5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7"/>
+      <c r="B6" s="5">
         <v>10020.0</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="F5" s="5">
+      <c r="C6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="5">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="2">
+      <c r="F6" s="5">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6"/>
+      <c r="B7" s="5">
         <v>10021.0</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F6" s="2">
-        <v>10.0</v>
+      <c r="C7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="5">
+        <v>12.0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>